<commit_message>
Added browser navigation and tab handling tests
</commit_message>
<xml_diff>
--- a/resources/data/LoginData.xlsx
+++ b/resources/data/LoginData.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raman\SeleniumAutomationFramework\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80D34E31-38C4-4460-87CC-36D024997601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3F168E-6D26-4D00-88DD-B0690C1F4F68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="12" windowWidth="11424" windowHeight="6444" xr2:uid="{48BD7C7A-5236-404F-9E04-25CEEB34BEC7}"/>
+    <workbookView xWindow="0" yWindow="12" windowWidth="11424" windowHeight="9012" xr2:uid="{48BD7C7A-5236-404F-9E04-25CEEB34BEC7}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>